<commit_message>
feat: Complete generation selector with dark mode, centered window, and integrated generation
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -668,8 +668,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>7</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -681,8 +683,10 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n">
-        <v>46083</v>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -700,6 +704,86 @@
         </is>
       </c>
       <c r="I4" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>10 000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46084</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>10 000</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -716,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1000,11 +1084,15 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B4" t="n">
-        <v>7</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1024,16 +1112,112 @@
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="4" t="n"/>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>M.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>M.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="N6" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O6" s="2" t="n">
         <v>100000</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1050,7 +1234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1190,14 +1374,20 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>46083</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1206,11 +1396,73 @@
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="8" t="n">
-        <v>46083</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>46083</v>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>46084</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="8" t="n">
+        <v>46084</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>46084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update project files
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,11 +512,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -752,8 +752,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>9</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -765,8 +767,10 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n">
-        <v>46084</v>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -784,6 +788,30 @@
         </is>
       </c>
       <c r="I6" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SOUFIANE OUMAS ET ZAHRA RAFIQ</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46085</v>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -800,20 +828,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="56" customWidth="1" min="11" max="11"/>
+    <col width="66" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="29" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
@@ -1184,11 +1212,15 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B6" t="n">
-        <v>9</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1208,16 +1240,93 @@
       </c>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="4" t="n"/>
-      <c r="N6" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>100000</v>
-      </c>
-      <c r="P6" t="n">
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>M.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SOUFIANE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OUMAS</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BL82562</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>14/05/2035</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>31552</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>LOT OLD HADDOU N 50 APT 05 ETG 03 SD HAJJAJ OD HASSAR TIT MELLIL</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>0661792201</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>soufiane.osf@gmail.com</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1234,7 +1343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1442,14 +1551,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>46084</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1458,11 +1573,43 @@
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="8" t="n">
-        <v>46084</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>46084</v>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>46085</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>46085</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>46816</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: migrate templates, database, and dashboard contract fields
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -514,60 +514,49 @@
   </sheetPr>
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="64" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>DEN_STE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>FORME_JUR</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>ICE</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>DATE_ICE</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>CAPITAL</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>PART_SOCIAL</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>STE_ADRESS</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>TRIBUNAL</t>
         </is>
@@ -594,12 +583,12 @@
           <t>003883436000057</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>2025-12-31 00:00:00</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
@@ -609,7 +598,7 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300, ETG 2, N 162, AIN CHOK CASABLANCA</t>
         </is>
@@ -641,12 +630,12 @@
           <t>003888708000012</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2026-01-09 00:00:00</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
@@ -656,7 +645,7 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA </t>
         </is>
@@ -683,12 +672,13 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -698,7 +688,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -725,12 +715,13 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -740,7 +731,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -767,12 +758,13 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -782,7 +774,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -794,19 +786,26 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>10</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>SOUFIANE OUMAS ET ZAHRA RAFIQ</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
-        <v>46085</v>
-      </c>
-      <c r="F7" s="2" t="n"/>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK</t>
         </is>
@@ -830,108 +829,89 @@
   </sheetPr>
   <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="66" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="29" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ID_ASSOCIE</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>PRENOM</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>NOM</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>NATIONALITY</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>CIN_NUM</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>CIN_VALIDATY</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>DATE_NAISS</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>LIEU_NAISS</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>ADRESSE</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>PHONE</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>PARTS</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>CAPITAL_DETENU</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>IS_GERANT</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="Q1" s="9" t="inlineStr">
         <is>
           <t>QUALITY</t>
         </is>
@@ -978,22 +958,22 @@
           <t>26/09/2029</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>1980-10-06 00:00:00</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>MERS SULTAN DERB SOLTANE AL FIDA</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>JNANE CALIFORNIE RES EMMERAUDE 9 APT 10 AIN CHOCK CASA</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>0661155849</t>
         </is>
@@ -1003,12 +983,12 @@
           <t>brahim.elkhattaby@gmail.com</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1065,22 +1045,22 @@
           <t>13/11/2033</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>1990-09-28 00:00:00</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Fes</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>6 RUE 07 HAY MANSOUR C D CASABLANCA</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0665949398</t>
         </is>
@@ -1090,12 +1070,12 @@
           <t>elbetiouiyoussef@gmail.com</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1127,25 +1107,30 @@
           <t>M.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1177,25 +1162,30 @@
           <t>M.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1227,25 +1217,30 @@
           <t>M.</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="4" t="n"/>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1262,11 +1257,15 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B7" t="n">
-        <v>10</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1298,20 +1297,22 @@
           <t>14/05/2035</t>
         </is>
       </c>
-      <c r="I7" s="8" t="n">
-        <v>31552</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1986-05-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>LOT OLD HADDOU N 50 APT 05 ETG 03 SD HAJJAJ OD HASSAR TIT MELLIL</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>0661792201</t>
         </is>
@@ -1321,10 +1322,12 @@
           <t>soufiane.osf@gmail.com</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" t="n">
-        <v>1</v>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1343,58 +1346,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ID_CONTRAT</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>DATE_CONTRAT</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
-        <is>
-          <t>PERIOD_DOMCIL</t>
-        </is>
-      </c>
-      <c r="E1" s="12" t="inlineStr">
-        <is>
-          <t>PRIX_CONTRAT</t>
-        </is>
-      </c>
-      <c r="F1" s="12" t="inlineStr">
-        <is>
-          <t>PRIX_INTERMEDIARE_CONTRAT</t>
-        </is>
-      </c>
-      <c r="G1" s="12" t="inlineStr">
-        <is>
-          <t>DOM_DATEDEB</t>
-        </is>
-      </c>
-      <c r="H1" s="12" t="inlineStr">
-        <is>
-          <t>DOM_DATEFIN</t>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>DUREE_CONTRAT_MOIS</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>LOYER_MENSUEL_TTC</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>FRAIS_INTERMEDIAIRE_CONTRAT</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>DATE_DEBUT_CONTRAT</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>DATE_FIN_CONTRAT</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>TAUX_TVA_POURCENT</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>LOYER_MENSUEL_HT</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>MONTANT_TOTAL_HT_CONTRAT</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>MONTANT_PACK_DEMARRAGE_TTC</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>LOYER_MENSUEL_PACK_DEMARRAGE_TTC</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>TYPE_RENOUVELLEMENT</t>
+        </is>
+      </c>
+      <c r="O1" s="9" t="inlineStr">
+        <is>
+          <t>TAUX_TVA_RENOUVELLEMENT_POURCENT</t>
+        </is>
+      </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>LOYER_MENSUEL_HT_RENOUVELLEMENT</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
+          <t>MONTANT_TOTAL_HT_RENOUVELLEMENT</t>
+        </is>
+      </c>
+      <c r="R1" s="9" t="inlineStr">
+        <is>
+          <t>LOYER_MENSUEL_RENOUVELLEMENT_TTC</t>
+        </is>
+      </c>
+      <c r="S1" s="9" t="inlineStr">
+        <is>
+          <t>LOYER_ANNUEL_RENOUVELLEMENT_TTC</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1457,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2026-01-09 00:00:00</t>
         </is>
@@ -1419,26 +1467,37 @@
           <t>24</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>69.44</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>2026-01-09 00:00:00</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2028-01-09 00:00:00</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1451,7 +1510,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>2026-01-10 00:00:00</t>
         </is>
@@ -1461,26 +1520,37 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>125</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>1800</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>2026-01-10 00:00:00</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2027-01-10 00:00:00</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1493,7 +1563,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
@@ -1503,18 +1573,29 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1527,7 +1608,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
@@ -1537,18 +1618,29 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1561,7 +1653,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
@@ -1571,46 +1663,82 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B7" t="n">
-        <v>10</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>46085</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:00:00</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>46085</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>46816</v>
-      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>83.33</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2028-03-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: reorganize root files and update contract/template mappings
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,51 +512,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="64" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>DEN_STE</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>FORME_JUR</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>ICE</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>DATE_ICE</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>CAPITAL</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>PART_SOCIAL</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>STE_ADRESS</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>TRIBUNAL</t>
         </is>
@@ -583,12 +594,12 @@
           <t>003883436000057</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>2025-12-31 00:00:00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
@@ -598,7 +609,7 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300, ETG 2, N 162, AIN CHOK CASABLANCA</t>
         </is>
@@ -630,12 +641,12 @@
           <t>003888708000012</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>2026-01-09 00:00:00</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
@@ -645,7 +656,7 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA </t>
         </is>
@@ -672,13 +683,12 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -688,7 +698,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -715,13 +725,12 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -731,7 +740,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -758,13 +767,12 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -774,7 +782,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -796,21 +804,56 @@
           <t>SOUFIANE OUMAS ET ZAHRA RAFIQ</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>2026-03-04 00:00:00</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
+      <c r="F7" s="2" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PERSONA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46088</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -827,91 +870,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="66" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="29" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>ID_ASSOCIE</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>PRENOM</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>NOM</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>NATIONALITY</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>CIN_NUM</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>CIN_VALIDATY</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>DATE_NAISS</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>LIEU_NAISS</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>ADRESSE</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>PHONE</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>PARTS</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>CAPITAL_DETENU</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>IS_GERANT</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>QUALITY</t>
         </is>
@@ -958,22 +1020,22 @@
           <t>26/09/2029</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>1980-10-06 00:00:00</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>MERS SULTAN DERB SOLTANE AL FIDA</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>JNANE CALIFORNIE RES EMMERAUDE 9 APT 10 AIN CHOCK CASA</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>0661155849</t>
         </is>
@@ -983,12 +1045,12 @@
           <t>brahim.elkhattaby@gmail.com</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1045,22 +1107,22 @@
           <t>13/11/2033</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>1990-09-28 00:00:00</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Fes</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>6 RUE 07 HAY MANSOUR C D CASABLANCA</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>0665949398</t>
         </is>
@@ -1070,12 +1132,12 @@
           <t>elbetiouiyoussef@gmail.com</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1107,30 +1169,25 @@
           <t>M.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1162,30 +1219,25 @@
           <t>M.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1217,30 +1269,25 @@
           <t>M.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
@@ -1297,22 +1344,22 @@
           <t>14/05/2035</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>1986-05-20 00:00:00</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>LOT OLD HADDOU N 50 APT 05 ETG 03 SD HAJJAJ OD HASSAR TIT MELLIL</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>0661792201</t>
         </is>
@@ -1322,14 +1369,54 @@
           <t>soufiane.osf@gmail.com</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="4" t="n"/>
+      <c r="N8" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1346,101 +1433,134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="33" customWidth="1" min="18" max="18"/>
+    <col width="33" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="33" customWidth="1" min="21" max="21"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>ID_CONTRAT</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>DATE_CONTRAT</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>DUREE_CONTRAT_MOIS</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>TYPE_CONTRAT_DOMICILIATION</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>TYPE_CONTRAT_DOMICILIATION_AUTRE</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_TTC</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>FRAIS_INTERMEDIAIRE_CONTRAT</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>DATE_DEBUT_CONTRAT</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>DATE_FIN_CONTRAT</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>TAUX_TVA_POURCENT</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_HT</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>MONTANT_TOTAL_HT_CONTRAT</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>MONTANT_PACK_DEMARRAGE_TTC</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_PACK_DEMARRAGE_TTC</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>TYPE_RENOUVELLEMENT</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>TAUX_TVA_RENOUVELLEMENT_POURCENT</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="R1" s="12" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_HT_RENOUVELLEMENT</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="S1" s="12" t="inlineStr">
         <is>
           <t>MONTANT_TOTAL_HT_RENOUVELLEMENT</t>
         </is>
       </c>
-      <c r="R1" s="9" t="inlineStr">
+      <c r="T1" s="12" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_RENOUVELLEMENT_TTC</t>
         </is>
       </c>
-      <c r="S1" s="9" t="inlineStr">
+      <c r="U1" s="12" t="inlineStr">
         <is>
           <t>LOYER_ANNUEL_RENOUVELLEMENT_TTC</t>
         </is>
@@ -1457,7 +1577,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>2026-01-09 00:00:00</t>
         </is>
@@ -1467,37 +1587,34 @@
           <t>24</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>69.44</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>2026-01-09 00:00:00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>2028-01-09 00:00:00</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="L2" s="5" t="n"/>
+      <c r="M2" s="5" t="n"/>
+      <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+      <c r="R2" s="5" t="n"/>
+      <c r="S2" s="5" t="n"/>
+      <c r="T2" s="5" t="n"/>
+      <c r="U2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1510,7 +1627,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>2026-01-10 00:00:00</t>
         </is>
@@ -1520,37 +1637,34 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>125</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>1800</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>2026-01-10 00:00:00</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>2027-01-10 00:00:00</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="n"/>
+      <c r="O3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
+      <c r="S3" s="5" t="n"/>
+      <c r="T3" s="5" t="n"/>
+      <c r="U3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1563,7 +1677,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
@@ -1573,29 +1687,26 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="n"/>
+      <c r="R4" s="5" t="n"/>
+      <c r="S4" s="5" t="n"/>
+      <c r="T4" s="5" t="n"/>
+      <c r="U4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1608,7 +1719,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
@@ -1618,29 +1729,26 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
+      <c r="R5" s="5" t="n"/>
+      <c r="S5" s="5" t="n"/>
+      <c r="T5" s="5" t="n"/>
+      <c r="U5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1653,7 +1761,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
@@ -1663,29 +1771,26 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>2026-03-03 00:00:00</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="5" t="n"/>
+      <c r="T6" s="5" t="n"/>
+      <c r="U6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1698,7 +1803,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>2026-03-04 00:00:00</t>
         </is>
@@ -1708,37 +1813,100 @@
           <t>24</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>83.33</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>2026-03-04 00:00:00</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>2028-03-04 00:00:00</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>46088</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Association</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="8" t="n">
+        <v>46088</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>46452</v>
+      </c>
+      <c r="K8" t="n">
+        <v>20</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>83.33329999999999</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>20</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>166.667</v>
+      </c>
+      <c r="S8" s="5" t="n">
+        <v>166.67</v>
+      </c>
+      <c r="T8" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="U8" s="5" t="n">
+        <v>2400</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
release: v2.2.2 defaults, activities UX, and generation improvements
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -522,8 +522,10 @@
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="64" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="64" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,10 +566,20 @@
       </c>
       <c r="H1" s="12" t="inlineStr">
         <is>
+          <t>VALEUR_NOMINALE</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>DATE_EXP_CERT_NEG</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
           <t>STE_ADRESS</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>TRIBUNAL</t>
         </is>
@@ -609,12 +621,13 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="8" t="n"/>
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300, ETG 2, N 162, AIN CHOK CASABLANCA</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -656,12 +669,13 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="8" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA </t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -698,12 +712,13 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -740,12 +755,13 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -782,12 +798,13 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -810,20 +827,23 @@
         </is>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>11</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -835,8 +855,10 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E8" s="8" t="n">
-        <v>46088</v>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-07 00:00:00</t>
+        </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -848,12 +870,319 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NOUVELLE STE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NOUVELLE STE1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NOUVELLE STE356</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NOUVELLE STE35</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Latrubine</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SANDALA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>46089</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>46089</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -870,7 +1199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -886,10 +1215,11 @@
     <col width="66" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="29" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -960,20 +1290,25 @@
       </c>
       <c r="N1" s="12" t="inlineStr">
         <is>
+          <t>PART_PERCENT</t>
+        </is>
+      </c>
+      <c r="O1" s="12" t="inlineStr">
+        <is>
           <t>PARTS</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>CAPITAL_DETENU</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>IS_GERANT</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="R1" s="12" t="inlineStr">
         <is>
           <t>QUALITY</t>
         </is>
@@ -1045,22 +1380,22 @@
           <t>brahim.elkhattaby@gmail.com</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1132,22 +1467,22 @@
           <t>elbetiouiyoussef@gmail.com</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1182,22 +1517,22 @@
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="4" t="n"/>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1232,22 +1567,22 @@
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="4" t="n"/>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1282,22 +1617,22 @@
       </c>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="4" t="n"/>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>100000</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1369,25 +1704,29 @@
           <t>soufiane.osf@gmail.com</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
-      <c r="P7" t="inlineStr">
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B8" t="n">
-        <v>11</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1407,16 +1746,400 @@
       </c>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="4" t="n"/>
-      <c r="N8" s="2" t="n">
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="4" t="n"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="4" t="n"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="4" t="n"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="4" t="n"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="4" t="n"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B14" t="n">
+        <v>17</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="N14" t="n">
+        <v>100</v>
+      </c>
+      <c r="O14" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="P14" s="2" t="n">
         <v>100000</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q14" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -1433,7 +2156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1843,14 +2566,20 @@
       <c r="U7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B8" t="n">
-        <v>11</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>46088</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-07 00:00:00</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1862,49 +2591,631 @@
           <t>Association</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>2027-03-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>2028-03-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B14" t="n">
+        <v>17</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>46089</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="8" t="n">
-        <v>46088</v>
-      </c>
-      <c r="J8" s="8" t="n">
-        <v>46452</v>
-      </c>
-      <c r="K8" t="n">
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="8" t="n">
+        <v>46089</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>46089</v>
+      </c>
+      <c r="K14" t="n">
         <v>20</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="L14" s="5" t="n">
         <v>83.33329999999999</v>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="M14" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="N14" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="O14" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Mensuel</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q14" t="n">
         <v>20</v>
       </c>
-      <c r="R8" s="5" t="n">
+      <c r="R14" s="5" t="n">
         <v>166.667</v>
       </c>
-      <c r="S8" s="5" t="n">
+      <c r="S14" s="5" t="n">
         <v>166.67</v>
       </c>
-      <c r="T8" s="5" t="n">
+      <c r="T14" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="U8" s="5" t="n">
+      <c r="U14" s="5" t="n">
         <v>2400</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update SARL template loops, signature mode, and defaults guide
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,13 +512,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -1143,8 +1143,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>17</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1156,33 +1158,145 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LA COMMUNE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SARL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0000000012555520</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SLAMA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SARL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0002551250022</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I16" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -1199,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1208,7 +1322,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
@@ -2093,11 +2207,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>18</v>
-      </c>
-      <c r="B14" t="n">
-        <v>17</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -2127,19 +2245,326 @@
       </c>
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="4" t="n"/>
-      <c r="N14" t="n">
-        <v>100</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>100000</v>
-      </c>
-      <c r="Q14" t="n">
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PRENOM1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NOM1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>BH5080122</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>SLOUMANA Rure casa Porat reico</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="n"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PRENOM2</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NOM2</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Cameronnie</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>COM15151JU</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>QEILOU DUR ALBAH RUE 25 N 15 CAME</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="n"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B17" t="n">
+        <v>19</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PRENOM1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>NOM1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>BH41516</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>47829</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>TOUJTAT AL AOUNATE RUE 15 DOUAR SAMIR</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="n"/>
+      <c r="N17" t="n">
+        <v>50</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="Q17" t="n">
         <v>1</v>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B18" t="n">
+        <v>19</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PRENOM2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NOM2</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Cameronnie</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CAM155OI</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>12/12/2031</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>36008</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>SOULIA ETUDE 12 ETG 1 CASA</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="n"/>
+      <c r="N18" t="n">
+        <v>50</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -2156,7 +2581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3154,68 +3579,264 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>17</v>
-      </c>
-      <c r="B14" t="n">
-        <v>17</v>
-      </c>
-      <c r="C14" s="8" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>2027-06-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U15" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B16" t="n">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G16" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="8" t="n">
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="J14" s="8" t="n">
-        <v>46089</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="J16" s="8" t="n">
+        <v>46545</v>
+      </c>
+      <c r="K16" t="n">
         <v>20</v>
       </c>
-      <c r="L14" s="5" t="n">
+      <c r="L16" s="5" t="n">
         <v>83.33329999999999</v>
       </c>
-      <c r="M14" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="O14" s="5" t="n">
+      <c r="M16" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="O16" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Mensuel</t>
         </is>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q16" t="n">
         <v>20</v>
       </c>
-      <c r="R14" s="5" t="n">
+      <c r="R16" s="5" t="n">
         <v>166.667</v>
       </c>
-      <c r="S14" s="5" t="n">
+      <c r="S16" s="5" t="n">
         <v>166.67</v>
       </c>
-      <c r="T14" s="5" t="n">
+      <c r="T16" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="U14" s="5" t="n">
+      <c r="U16" s="5" t="n">
         <v>2400</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: harmonize toolbar actions and move document generator to tools
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1252,8 +1252,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>19</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1270,33 +1272,83 @@
           <t>0002551250022</t>
         </is>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NOND</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I17" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
@@ -1313,7 +1365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2433,11 +2485,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>21</v>
-      </c>
-      <c r="B17" t="n">
-        <v>19</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2469,8 +2525,10 @@
           <t>08/03/2026</t>
         </is>
       </c>
-      <c r="I17" s="8" t="n">
-        <v>47829</v>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>2030-12-12 00:00:00</t>
+        </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
@@ -2483,88 +2541,163 @@
         </is>
       </c>
       <c r="L17" s="4" t="n"/>
-      <c r="N17" t="n">
-        <v>50</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="P17" s="2" t="n">
-        <v>50000</v>
-      </c>
-      <c r="Q17" t="n">
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PRENOM2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NOM2</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Cameronnie</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CAM155OI</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>12/12/2031</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>1998-08-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>SOULIA ETUDE 12 ETG 1 CASA</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="n"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Associé Gérant</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>23</v>
+      </c>
+      <c r="B19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="4" t="n"/>
+      <c r="N19" t="n">
+        <v>100</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="Q19" t="n">
         <v>1</v>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Associé Gérant</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>22</v>
-      </c>
-      <c r="B18" t="n">
-        <v>19</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Monsieur</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>PRENOM2</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>NOM2</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Cameronnie</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>CAM155OI</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>12/12/2031</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="n">
-        <v>36008</v>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Casablanca</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>SOULIA ETUDE 12 ETG 1 CASA</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="n"/>
-      <c r="N18" t="n">
-        <v>50</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="P18" s="2" t="n">
-        <v>50000</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>1</v>
-      </c>
-      <c r="R18" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>Associé Gérant</t>
         </is>
@@ -2581,7 +2714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3775,68 +3908,166 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>19</v>
-      </c>
-      <c r="B16" t="n">
-        <v>19</v>
-      </c>
-      <c r="C16" s="8" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>2027-06-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>83.3333</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>166.667</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>166.67</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="U16" s="5" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C17" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="G17" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="8" t="n">
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="8" t="n">
         <v>46089</v>
       </c>
-      <c r="J16" s="8" t="n">
-        <v>46545</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="J17" s="8" t="n">
+        <v>46453</v>
+      </c>
+      <c r="K17" t="n">
         <v>20</v>
       </c>
-      <c r="L16" s="5" t="n">
+      <c r="L17" s="5" t="n">
         <v>83.33329999999999</v>
       </c>
-      <c r="M16" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N16" s="5" t="n">
-        <v>1500</v>
-      </c>
-      <c r="O16" s="5" t="n">
+      <c r="M17" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="O17" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>Mensuel</t>
         </is>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>20</v>
       </c>
-      <c r="R16" s="5" t="n">
+      <c r="R17" s="5" t="n">
         <v>166.667</v>
       </c>
-      <c r="S16" s="5" t="n">
+      <c r="S17" s="5" t="n">
         <v>166.67</v>
       </c>
-      <c r="T16" s="5" t="n">
+      <c r="T17" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="U16" s="5" t="n">
+      <c r="U17" s="5" t="n">
         <v>2400</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: finalize dashboard and form formatting improvements
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -512,76 +512,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="64" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>DEN_STE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>FORME_JUR</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>ICE</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>DATE_ICE</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>CAPITAL</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>PART_SOCIAL</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>VALEUR_NOMINALE</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>DATE_EXP_CERT_NEG</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>STE_ADRESS</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>TRIBUNAL</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>TYPE_GENERATION</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>PROCEDURE_CREATION</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>MODE_DEPOT_CREATION</t>
         </is>
       </c>
     </row>
@@ -606,23 +608,24 @@
           <t>003883436000057</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>2025-12-31 00:00:00</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>31/12/2025</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I2" s="8" t="n"/>
-      <c r="J2" s="3" t="inlineStr">
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300, ETG 2, N 162, AIN CHOK CASABLANCA</t>
         </is>
@@ -632,6 +635,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -654,25 +660,26 @@
           <t>003888708000012</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>2026-01-09 00:00:00</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="n"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA </t>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -680,6 +687,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -697,12 +707,13 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-02 00:00:00</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -712,8 +723,9 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -723,6 +735,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -740,12 +755,13 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -755,8 +771,9 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -766,6 +783,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -783,12 +803,13 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>10 000</t>
         </is>
@@ -798,8 +819,9 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>46 BD ZERKTOUNI ETG 2 APPT 6 CASABLANCA</t>
         </is>
@@ -809,6 +831,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -821,14 +846,18 @@
           <t>SOUFIANE OUMAS ET ZAHRA RAFIQ</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-04 00:00:00</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK</t>
         </is>
@@ -838,6 +867,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -855,23 +887,25 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-07 00:00:00</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="3" t="inlineStr">
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -881,6 +915,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -898,19 +935,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -918,12 +956,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -933,6 +971,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -950,19 +991,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -970,12 +1012,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -985,6 +1027,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1002,19 +1047,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1022,12 +1068,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1037,6 +1083,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1054,19 +1103,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1074,12 +1124,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1089,6 +1139,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1106,19 +1159,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1126,12 +1180,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1141,6 +1195,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1158,19 +1215,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1178,12 +1236,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1193,6 +1251,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1215,19 +1276,19 @@
           <t>0000000012555520</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1235,12 +1296,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1250,6 +1311,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1272,19 +1336,19 @@
           <t>0002551250022</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1292,12 +1356,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1307,10 +1371,15 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>20</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1322,17 +1391,20 @@
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n">
-        <v>46089</v>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1340,10 +1412,12 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I17" s="8" t="n">
-        <v>46089</v>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
@@ -1353,6 +1427,9 @@
           <t>Casablanca</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1367,114 +1444,94 @@
   </sheetPr>
   <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="66" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="29" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ID_ASSOCIE</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>PRENOM</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>NOM</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>NATIONALITY</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>CIN_NUM</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>CIN_VALIDATY</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>DATE_NAISS</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>LIEU_NAISS</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>ADRESSE</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>PHONE</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>PART_PERCENT</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>PARTS</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>CAPITAL_DETENU</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="Q1" s="9" t="inlineStr">
         <is>
           <t>IS_GERANT</t>
         </is>
       </c>
-      <c r="R1" s="12" t="inlineStr">
+      <c r="R1" s="9" t="inlineStr">
         <is>
           <t>QUALITY</t>
         </is>
@@ -1521,22 +1578,22 @@
           <t>26/09/2029</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>1980-10-06 00:00:00</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>10/06/1980</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>MERS SULTAN DERB SOLTANE AL FIDA</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>JNANE CALIFORNIE RES EMMERAUDE 9 APT 10 AIN CHOCK CASA</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>0661155849</t>
         </is>
@@ -1546,19 +1603,20 @@
           <t>brahim.elkhattaby@gmail.com</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -1608,22 +1666,22 @@
           <t>13/11/2033</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>1990-09-28 00:00:00</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28/09/1990</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Fes</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>6 RUE 07 HAY MANSOUR C D CASABLANCA</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0665949398</t>
         </is>
@@ -1633,19 +1691,20 @@
           <t>elbetiouiyoussef@gmail.com</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1670,32 +1729,38 @@
           <t>M.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -1720,32 +1785,38 @@
           <t>M.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1770,32 +1841,38 @@
           <t>M.</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="4" t="n"/>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1845,22 +1922,22 @@
           <t>14/05/2035</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>1986-05-20 00:00:00</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>20/05/1986</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>LOT OLD HADDOU N 50 APT 05 ETG 03 SD HAJJAJ OD HASSAR TIT MELLIL</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>0661792201</t>
         </is>
@@ -1870,11 +1947,12 @@
           <t>soufiane.osf@gmail.com</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1899,32 +1977,38 @@
           <t>Monsieur</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1964,32 +2048,35 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="4" t="n"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -2029,32 +2116,35 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="4" t="n"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -2094,32 +2184,35 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="4" t="n"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -2159,32 +2252,35 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="4" t="n"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -2224,32 +2320,35 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="4" t="n"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -2289,32 +2388,35 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I14" s="8" t="n"/>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="4" t="n"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>100000</t>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>100 000</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -2359,40 +2461,42 @@
           <t>BH5080122</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-04 00:00:00</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>SLOUMANA Rure casa Porat reico</t>
         </is>
       </c>
-      <c r="L15" s="4" t="n"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>50000</t>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>50 000</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2442,40 +2546,41 @@
           <t>12/03/2026</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-02 00:00:00</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>QEILOU DUR ALBAH RUE 25 N 15 CAME</t>
         </is>
       </c>
-      <c r="L16" s="4" t="n"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>50000</t>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>50 000</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2525,40 +2630,41 @@
           <t>08/03/2026</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>2030-12-12 00:00:00</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>12/12/2030</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>TOUJTAT AL AOUNATE RUE 15 DOUAR SAMIR</t>
         </is>
       </c>
-      <c r="L17" s="4" t="n"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>50000</t>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>50 000</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2608,40 +2714,41 @@
           <t>12/12/2031</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>1998-08-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>08/01/1998</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>SOULIA ETUDE 12 ETG 1 CASA</t>
         </is>
       </c>
-      <c r="L18" s="4" t="n"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>50000</t>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>50 000</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2651,11 +2758,15 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>23</v>
-      </c>
-      <c r="B19" t="n">
-        <v>20</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2677,25 +2788,36 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="N19" t="n">
-        <v>100</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="P19" s="2" t="n">
-        <v>100000</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>1</v>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -2716,132 +2838,109 @@
   </sheetPr>
   <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="29" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="33" customWidth="1" min="18" max="18"/>
-    <col width="33" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
-    <col width="33" customWidth="1" min="21" max="21"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ID_CONTRAT</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>ID_SOCIETE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>DATE_CONTRAT</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>DUREE_CONTRAT_MOIS</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>TYPE_CONTRAT_DOMICILIATION</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>TYPE_CONTRAT_DOMICILIATION_AUTRE</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_TTC</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>FRAIS_INTERMEDIAIRE_CONTRAT</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>DATE_DEBUT_CONTRAT</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>DATE_FIN_CONTRAT</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>TAUX_TVA_POURCENT</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_HT</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>MONTANT_TOTAL_HT_CONTRAT</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>MONTANT_PACK_DEMARRAGE_TTC</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_PACK_DEMARRAGE_TTC</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>TYPE_RENOUVELLEMENT</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="Q1" s="9" t="inlineStr">
         <is>
           <t>TAUX_TVA_RENOUVELLEMENT_POURCENT</t>
         </is>
       </c>
-      <c r="R1" s="12" t="inlineStr">
+      <c r="R1" s="9" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_HT_RENOUVELLEMENT</t>
         </is>
       </c>
-      <c r="S1" s="12" t="inlineStr">
+      <c r="S1" s="9" t="inlineStr">
         <is>
           <t>MONTANT_TOTAL_HT_RENOUVELLEMENT</t>
         </is>
       </c>
-      <c r="T1" s="12" t="inlineStr">
+      <c r="T1" s="9" t="inlineStr">
         <is>
           <t>LOYER_MENSUEL_RENOUVELLEMENT_TTC</t>
         </is>
       </c>
-      <c r="U1" s="12" t="inlineStr">
+      <c r="U1" s="9" t="inlineStr">
         <is>
           <t>LOYER_ANNUEL_RENOUVELLEMENT_TTC</t>
         </is>
@@ -2858,9 +2957,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>2026-01-09 00:00:00</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2868,34 +2967,39 @@
           <t>24</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>69.44</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>2026-01-09 00:00:00</t>
-        </is>
-      </c>
-      <c r="J2" s="8" t="inlineStr">
-        <is>
-          <t>2028-01-09 00:00:00</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="n"/>
-      <c r="N2" s="5" t="n"/>
-      <c r="O2" s="5" t="n"/>
-      <c r="R2" s="5" t="n"/>
-      <c r="S2" s="5" t="n"/>
-      <c r="T2" s="5" t="n"/>
-      <c r="U2" s="5" t="n"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>69,44</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>01/09/2028</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2908,9 +3012,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>2026-01-10 00:00:00</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2918,34 +3022,39 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>1800</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>2026-01-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>2027-01-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
-      <c r="N3" s="5" t="n"/>
-      <c r="O3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
-      <c r="S3" s="5" t="n"/>
-      <c r="T3" s="5" t="n"/>
-      <c r="U3" s="5" t="n"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1 800,00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>01/10/2027</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2958,9 +3067,9 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-02 00:00:00</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2968,26 +3077,31 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-02 00:00:00</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-02 00:00:00</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3000,9 +3114,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3010,26 +3124,31 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
-      <c r="S5" s="5" t="n"/>
-      <c r="T5" s="5" t="n"/>
-      <c r="U5" s="5" t="n"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3042,9 +3161,9 @@
           <t>9</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3052,26 +3171,31 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03 00:00:00</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
-      <c r="T6" s="5" t="n"/>
-      <c r="U6" s="5" t="n"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3084,9 +3208,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-04 00:00:00</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3094,34 +3218,39 @@
           <t>24</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>83.33</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-04 00:00:00</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>2028-03-04 00:00:00</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>83,33</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>03/04/2028</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3134,9 +3263,9 @@
           <t>11</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-07 00:00:00</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3149,20 +3278,21 @@
           <t>Association</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-07 00:00:00</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>2027-03-06 00:00:00</t>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>03/06/2027</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3170,24 +3300,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -3200,24 +3330,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R8" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S8" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U8" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3232,9 +3362,9 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3247,20 +3377,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3268,24 +3399,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -3298,24 +3429,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R9" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S9" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T9" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U9" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3330,9 +3461,9 @@
           <t>13</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -3345,20 +3476,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>2028-03-07 00:00:00</t>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>03/07/2028</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3366,24 +3498,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -3396,24 +3528,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R10" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3428,9 +3560,9 @@
           <t>14</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3443,20 +3575,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3464,24 +3597,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -3494,24 +3627,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R11" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S11" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3526,9 +3659,9 @@
           <t>15</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -3541,20 +3674,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -3562,24 +3696,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -3592,24 +3726,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R12" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S12" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U12" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3624,9 +3758,9 @@
           <t>16</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3639,20 +3773,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -3660,24 +3795,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -3690,24 +3825,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R13" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T13" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3722,9 +3857,9 @@
           <t>17</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -3737,20 +3872,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -3758,24 +3894,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -3788,24 +3924,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R14" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S14" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U14" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3820,9 +3956,9 @@
           <t>18</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3835,20 +3971,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>2027-06-07 00:00:00</t>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>06/07/2027</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -3856,24 +3993,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
-        <is>
-          <t>1250</t>
-        </is>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="O15" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>1 250,00</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>1 500,00</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3886,24 +4023,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R15" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S15" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T15" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U15" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
@@ -3918,9 +4055,9 @@
           <t>19</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -3933,20 +4070,21 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>2027-06-07 00:00:00</t>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>06/07/2027</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -3954,24 +4092,24 @@
           <t>20</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>83.3333</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
-        <is>
-          <t>1250</t>
-        </is>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>1 250,00</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>1 500,00</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>100,00</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3984,36 +4122,42 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R16" s="5" t="inlineStr">
-        <is>
-          <t>166.667</t>
-        </is>
-      </c>
-      <c r="S16" s="5" t="inlineStr">
-        <is>
-          <t>166.67</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="U16" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>20</v>
-      </c>
-      <c r="B17" t="n">
-        <v>20</v>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>46089</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -4025,50 +4169,77 @@
           <t>Personne Morale</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="8" t="n">
-        <v>46089</v>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>46453</v>
-      </c>
-      <c r="K17" t="n">
-        <v>20</v>
-      </c>
-      <c r="L17" s="5" t="n">
-        <v>83.33329999999999</v>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="N17" s="5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="O17" s="5" t="n">
-        <v>100</v>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>03/07/2027</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
           <t>Mensuel</t>
         </is>
       </c>
-      <c r="Q17" t="n">
-        <v>20</v>
-      </c>
-      <c r="R17" s="5" t="n">
-        <v>166.667</v>
-      </c>
-      <c r="S17" s="5" t="n">
-        <v>166.67</v>
-      </c>
-      <c r="T17" s="5" t="n">
-        <v>200</v>
-      </c>
-      <c r="U17" s="5" t="n">
-        <v>2400</v>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>166,67</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: generation edit flow and output prompt
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,65 +524,70 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
+          <t>N° dossier domiciliation</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
           <t>Dénomination sociale</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>forme_jur</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>ice</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>date_ice</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>capital</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>part_social</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>valeur_nominale</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>date_exp_cert_neg</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>ste_adress</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>tribunal</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>type_generation</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>procedure_creation</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>mode_depot_creation</t>
         </is>
@@ -594,52 +599,290 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>NOUVELLE STE</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>SARL AU</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>13/03/2026</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>1 000</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>creation</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOM-0011</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SUCCURSALE SIEGALE 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SARL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>003941457000040</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>domiciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOM-0012</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pooppp</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>domiciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ITISSSALAT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>creation</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ITISSSALAT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SARL AU</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>creation</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
@@ -656,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,6 +1061,371 @@
         </is>
       </c>
       <c r="S2" t="inlineStr">
+        <is>
+          <t>Associé</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SUCCURSALE SIEGALE 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Madame</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AOUATIF</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>HALIOUA</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>F748671</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>16/04/2028</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>01/12/1990</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>DIOUR LAKRAM RUE 6 NR 23 MOHAMMEDIA</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0631160987</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>A.HALIOUA@ARTEX-BUSINESS.COM</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Associé</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SUCCURSALE SIEGALE 2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Associé</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>pooppp</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Associé</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ITISSSALAT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Associé</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ITISSSALAT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
         <is>
           <t>Associé</t>
         </is>
@@ -834,7 +1442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1046,6 +1654,414 @@
         </is>
       </c>
       <c r="V2" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SUCCURSALE SIEGALE 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>600,00</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Annuel</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pooppp</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>01/04/2027</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Annuel</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ITISSSALAT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>01/04/2027</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Annuel</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ITISSSALAT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>01/04/2027</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1 000,00</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>1 200,00</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Annuel</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>2 400,00</t>
         </is>
@@ -1062,7 +2078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1191,6 +2207,33 @@
       <c r="M2" t="inlineStr">
         <is>
           <t>fid.basma@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>COAG -- Coursier Comptable Agréé</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>COAG</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>YOUSSEF</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0660002741</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: associe roles defaults and dashboard columns
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,22 +596,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DOM-0011</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NOUVELLE STE</t>
+          <t>SUCCURSALE SIEGALE 2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SARL AU</t>
+          <t>SARL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>003941457000040</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -629,6 +639,11 @@
           <t>100</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
@@ -641,44 +656,34 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>creation</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>normal</t>
+          <t>domiciliation</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DOM-0011</t>
+          <t>DOM-0012</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SUCCURSALE SIEGALE 2</t>
+          <t>pooppp</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SARL</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>003941457000040</t>
+          <t>SARL AU</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -694,11 +699,6 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>100</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>30/06/2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -720,17 +720,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DOM-0012</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pooppp</t>
+          <t>IWAN TEC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -738,9 +733,14 @@
           <t>SARL AU</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>00001251256500255</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -758,6 +758,11 @@
           <t>100</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>25/12/2029</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
@@ -770,119 +775,10 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>domiciliation</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ITISSSALAT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SARL AU</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>100 000</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>1 000</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Casablanca</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
           <t>creation</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ITISSSALAT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SARL AU</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>100 000</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>1 000</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Casablanca</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>creation</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
@@ -899,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1002,32 +898,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NOUVELLE STE</t>
+          <t>SUCCURSALE SIEGALE 2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Monsieur</t>
+          <t>Madame</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PRENOM</t>
+          <t>AOUATIF</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NOM</t>
+          <t>HALIOUA</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1035,9 +931,39 @@
           <t>Marocaine</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>F748671</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>16/04/2028</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>01/12/1990</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>DIOUR LAKRAM RUE 6 NR 23 MOHAMMEDIA</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0631160987</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>A.HALIOUA@ARTEX-BUSINESS.COM</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1069,14 +995,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>SUCCURSALE SIEGALE 2</t>
@@ -1084,17 +1010,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Madame</t>
+          <t>Monsieur</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AOUATIF</t>
+          <t>PRENOM</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>HALIOUA</t>
+          <t>NOM</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1102,54 +1028,24 @@
           <t>Marocaine</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>F748671</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>16/04/2028</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>01/12/1990</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>DIOUR LAKRAM RUE 6 NR 23 MOHAMMEDIA</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0631160987</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>A.HALIOUA@ARTEX-BUSINESS.COM</t>
-        </is>
-      </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1 000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>100 000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1166,17 +1062,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SUCCURSALE SIEGALE 2</t>
+          <t>pooppp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1206,17 +1102,17 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1 000</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100 000</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -1233,17 +1129,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pooppp</t>
+          <t>IWAN TEC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1253,12 +1149,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PRENOM</t>
+          <t>SOUHAM</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>NOM</t>
+          <t>ABID</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1266,6 +1162,21 @@
           <t>Marocaine</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NH1841</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>12/04/2030</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>10/12/1992</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Casablanca</t>
@@ -1292,140 +1203,6 @@
         </is>
       </c>
       <c r="S5" t="inlineStr">
-        <is>
-          <t>Associé</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ITISSSALAT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Monsieur</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>PRENOM</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>NOM</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Marocaine</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Casablanca</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>1 000</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>100 000</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Associé</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ITISSSALAT</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Monsieur</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>PRENOM</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>NOM</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Marocaine</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Casablanca</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>1 000</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>100 000</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
         <is>
           <t>Associé</t>
         </is>
@@ -1442,7 +1219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1560,27 +1337,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NOUVELLE STE</t>
+          <t>SUCCURSALE SIEGALE 2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1595,12 +1372,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>12/03/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1615,12 +1392,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1 000,00</t>
+          <t>500,00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1 200,00</t>
+          <t>600,00</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -1662,27 +1439,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SUCCURSALE SIEGALE 2</t>
+          <t>pooppp</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1697,12 +1474,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>01/04/2027</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1717,12 +1494,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>500,00</t>
+          <t>1 000,00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>600,00</t>
+          <t>1 200,00</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1764,22 +1541,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pooppp</t>
+          <t>IWAN TEC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1799,12 +1576,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>01/04/2027</t>
+          <t>03/04/2027</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1858,210 +1635,6 @@
         </is>
       </c>
       <c r="V4" t="inlineStr">
-        <is>
-          <t>2 400,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ITISSSALAT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Personne Morale</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>100,00</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>01/04/2027</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>83,3333</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1 000,00</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>1 200,00</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>100,00</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Annuel</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>166,667</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>2 000,00</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>200,00</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>2 400,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ITISSSALAT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Personne Morale</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>100,00</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>01/04/2027</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>83,3333</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>1 000,00</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>1 200,00</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>100,00</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Annuel</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>166,667</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>2 000,00</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>200,00</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
         <is>
           <t>2 400,00</t>
         </is>

</xml_diff>

<commit_message>
fix: improve startup fullscreen and dashboard window behavior on macOS
</commit_message>
<xml_diff>
--- a/databases/DataBase_domiciliation.xlsx
+++ b/databases/DataBase_domiciliation.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -781,6 +781,63 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOM-0013</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NOUv TEST</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SARL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>HAY MOULAY ABDELLAH RUE 300 N 152 ETG 2 AIN CHOCK, CASABLANCA</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>domiciliation</t>
         </is>
       </c>
     </row>
@@ -795,7 +852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -871,27 +928,27 @@
       </c>
       <c r="O1" s="9" t="inlineStr">
         <is>
+          <t>Qualité associé</t>
+        </is>
+      </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>Qualité gérant</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
           <t>part_percent</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="R1" s="9" t="inlineStr">
         <is>
           <t>parts</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="S1" s="9" t="inlineStr">
         <is>
           <t>capital_detenu</t>
-        </is>
-      </c>
-      <c r="R1" s="9" t="inlineStr">
-        <is>
-          <t>is_gerant</t>
-        </is>
-      </c>
-      <c r="S1" s="9" t="inlineStr">
-        <is>
-          <t>quality</t>
         </is>
       </c>
     </row>
@@ -966,29 +1023,19 @@
           <t>A.HALIOUA@ARTEX-BUSINESS.COM</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>1 000</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>100 000</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Associé</t>
         </is>
       </c>
     </row>
@@ -1033,29 +1080,19 @@
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Associé</t>
         </is>
       </c>
     </row>
@@ -1100,29 +1137,19 @@
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1 000</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>100 000</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Associé</t>
         </is>
       </c>
     </row>
@@ -1182,29 +1209,133 @@
           <t>Casablanca</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1 000</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>100 000</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Associé</t>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NOUv TEST</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1 000</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>100 000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>NOUv TEST</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Monsieur</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PRENOM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Marocaine</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1635,6 +1766,108 @@
         </is>
       </c>
       <c r="V4" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NOUv TEST</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Personne Morale</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>03/05/2028</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>83,3333</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2 400,00</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Annuel</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>166,667</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2 000,00</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>2 400,00</t>
         </is>

</xml_diff>